<commit_message>
feat: add user admin and refine brand controls
</commit_message>
<xml_diff>
--- a/docs/14-operations/templates/Teelle_Game_Review_Template_v2.xlsx
+++ b/docs/14-operations/templates/Teelle_Game_Review_Template_v2.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="بازی‌ها" sheetId="1" r:id="R4c06ef4bfc08436a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="بازی‌ها" sheetId="1" r:id="R05645816557a4e33"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -231,8 +231,8 @@
     <x:tableColumn id="7" name="موارد منع؛ با | جدا شوند"/>
     <x:tableColumn id="8" name="سطح نظارت"/>
     <x:tableColumn id="9" name="بازه سنی"/>
-    <x:tableColumn id="10" name="شروع سن به ماه"/>
-    <x:tableColumn id="11" name="پایان سن به ماه؛ غیرشامل"/>
+    <x:tableColumn id="10" name="شروع سن"/>
+    <x:tableColumn id="11" name="پایان سن"/>
     <x:tableColumn id="12" name="حداقل زمان؛ دقیقه"/>
     <x:tableColumn id="13" name="حداکثر زمان؛ دقیقه"/>
     <x:tableColumn id="14" name="زمان آماده‌سازی؛ دقیقه"/>
@@ -598,7 +598,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="6" t="str">
-        <x:v>هر بازی یک ردیف است. برای انتخاب چند گزینه، ستون‌های شماره‌دار کنار هم را پر کنید. پایان سن غیرشامل است؛ مثلاً ۲۴ یعنی تا پیش از ۲۴ماهگی.</x:v>
+        <x:v>هر بازی یک ردیف است. برای انتخاب چند گزینه، ستون‌های شماره‌دار کنار هم را پر کنید. سن، زمان، تعداد بازیکنان و همه گزینه‌های ثابت از منوی کشویی انتخاب می‌شوند.</x:v>
       </x:c>
       <x:c r="B2" s="6"/>
       <x:c r="C2" s="6"/>
@@ -855,10 +855,10 @@
         <x:v>بازه سنی</x:v>
       </x:c>
       <x:c r="J4" s="26" t="str">
-        <x:v>شروع سن به ماه</x:v>
+        <x:v>شروع سن</x:v>
       </x:c>
       <x:c r="K4" s="26" t="str">
-        <x:v>پایان سن به ماه؛ غیرشامل</x:v>
+        <x:v>پایان سن</x:v>
       </x:c>
       <x:c r="L4" s="27" t="str">
         <x:v>حداقل زمان؛ دقیقه</x:v>
@@ -1022,11 +1022,11 @@
       <x:c r="I5" s="32" t="str">
         <x:v>۶ تا ۲۳ ماه</x:v>
       </x:c>
-      <x:c r="J5" s="32" t="n">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="K5" s="32" t="n">
-        <x:v>24</x:v>
+      <x:c r="J5" s="32" t="str">
+        <x:v>۶ ماه</x:v>
+      </x:c>
+      <x:c r="K5" s="32" t="str">
+        <x:v>۲ سال</x:v>
       </x:c>
       <x:c r="L5" s="32" t="n">
         <x:v>3</x:v>
@@ -1160,11 +1160,11 @@
       <x:c r="I6" s="32" t="str">
         <x:v>۶ تا ۲۳ ماه</x:v>
       </x:c>
-      <x:c r="J6" s="32" t="n">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="K6" s="32" t="n">
-        <x:v>24</x:v>
+      <x:c r="J6" s="32" t="str">
+        <x:v>۶ ماه</x:v>
+      </x:c>
+      <x:c r="K6" s="32" t="str">
+        <x:v>۲ سال</x:v>
       </x:c>
       <x:c r="L6" s="32" t="n">
         <x:v>3</x:v>
@@ -1298,11 +1298,11 @@
       <x:c r="I7" s="32" t="str">
         <x:v>۶ تا ۲۳ ماه</x:v>
       </x:c>
-      <x:c r="J7" s="32" t="n">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="K7" s="32" t="n">
-        <x:v>24</x:v>
+      <x:c r="J7" s="32" t="str">
+        <x:v>۶ ماه</x:v>
+      </x:c>
+      <x:c r="K7" s="32" t="str">
+        <x:v>۲ سال</x:v>
       </x:c>
       <x:c r="L7" s="32" t="n">
         <x:v>3</x:v>
@@ -1436,11 +1436,11 @@
       <x:c r="I8" s="32" t="str">
         <x:v>۶ تا ۲۳ ماه</x:v>
       </x:c>
-      <x:c r="J8" s="32" t="n">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="K8" s="32" t="n">
-        <x:v>24</x:v>
+      <x:c r="J8" s="32" t="str">
+        <x:v>۶ ماه</x:v>
+      </x:c>
+      <x:c r="K8" s="32" t="str">
+        <x:v>۲ سال</x:v>
       </x:c>
       <x:c r="L8" s="32" t="n">
         <x:v>3</x:v>
@@ -1574,11 +1574,11 @@
       <x:c r="I9" s="32" t="str">
         <x:v>۶ تا ۲۳ ماه</x:v>
       </x:c>
-      <x:c r="J9" s="32" t="n">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="K9" s="32" t="n">
-        <x:v>24</x:v>
+      <x:c r="J9" s="32" t="str">
+        <x:v>۶ ماه</x:v>
+      </x:c>
+      <x:c r="K9" s="32" t="str">
+        <x:v>۲ سال</x:v>
       </x:c>
       <x:c r="L9" s="32" t="n">
         <x:v>3</x:v>
@@ -1712,11 +1712,11 @@
       <x:c r="I10" s="32" t="str">
         <x:v>۲ تا ۳ سال</x:v>
       </x:c>
-      <x:c r="J10" s="32" t="n">
-        <x:v>24</x:v>
-      </x:c>
-      <x:c r="K10" s="32" t="n">
-        <x:v>48</x:v>
+      <x:c r="J10" s="32" t="str">
+        <x:v>۲ سال</x:v>
+      </x:c>
+      <x:c r="K10" s="32" t="str">
+        <x:v>۴ سال</x:v>
       </x:c>
       <x:c r="L10" s="32" t="n">
         <x:v>5</x:v>
@@ -1856,11 +1856,11 @@
       <x:c r="I11" s="32" t="str">
         <x:v>۲ تا ۳ سال</x:v>
       </x:c>
-      <x:c r="J11" s="32" t="n">
-        <x:v>24</x:v>
-      </x:c>
-      <x:c r="K11" s="32" t="n">
-        <x:v>48</x:v>
+      <x:c r="J11" s="32" t="str">
+        <x:v>۲ سال</x:v>
+      </x:c>
+      <x:c r="K11" s="32" t="str">
+        <x:v>۴ سال</x:v>
       </x:c>
       <x:c r="L11" s="32" t="n">
         <x:v>5</x:v>
@@ -1998,11 +1998,11 @@
       <x:c r="I12" s="32" t="str">
         <x:v>۲ تا ۳ سال</x:v>
       </x:c>
-      <x:c r="J12" s="32" t="n">
-        <x:v>24</x:v>
-      </x:c>
-      <x:c r="K12" s="32" t="n">
-        <x:v>48</x:v>
+      <x:c r="J12" s="32" t="str">
+        <x:v>۲ سال</x:v>
+      </x:c>
+      <x:c r="K12" s="32" t="str">
+        <x:v>۴ سال</x:v>
       </x:c>
       <x:c r="L12" s="32" t="n">
         <x:v>5</x:v>
@@ -2136,11 +2136,11 @@
       <x:c r="I13" s="32" t="str">
         <x:v>۲ تا ۳ سال</x:v>
       </x:c>
-      <x:c r="J13" s="32" t="n">
-        <x:v>24</x:v>
-      </x:c>
-      <x:c r="K13" s="32" t="n">
-        <x:v>48</x:v>
+      <x:c r="J13" s="32" t="str">
+        <x:v>۲ سال</x:v>
+      </x:c>
+      <x:c r="K13" s="32" t="str">
+        <x:v>۴ سال</x:v>
       </x:c>
       <x:c r="L13" s="32" t="n">
         <x:v>5</x:v>
@@ -2276,11 +2276,11 @@
       <x:c r="I14" s="32" t="str">
         <x:v>۲ تا ۳ سال</x:v>
       </x:c>
-      <x:c r="J14" s="32" t="n">
-        <x:v>24</x:v>
-      </x:c>
-      <x:c r="K14" s="32" t="n">
-        <x:v>48</x:v>
+      <x:c r="J14" s="32" t="str">
+        <x:v>۲ سال</x:v>
+      </x:c>
+      <x:c r="K14" s="32" t="str">
+        <x:v>۴ سال</x:v>
       </x:c>
       <x:c r="L14" s="32" t="n">
         <x:v>6</x:v>
@@ -2420,11 +2420,11 @@
       <x:c r="I15" s="32" t="str">
         <x:v>۴ تا ۶ سال</x:v>
       </x:c>
-      <x:c r="J15" s="32" t="n">
-        <x:v>48</x:v>
-      </x:c>
-      <x:c r="K15" s="32" t="n">
-        <x:v>84</x:v>
+      <x:c r="J15" s="32" t="str">
+        <x:v>۴ سال</x:v>
+      </x:c>
+      <x:c r="K15" s="32" t="str">
+        <x:v>۷ سال</x:v>
       </x:c>
       <x:c r="L15" s="32" t="n">
         <x:v>6</x:v>
@@ -2562,11 +2562,11 @@
       <x:c r="I16" s="32" t="str">
         <x:v>۴ تا ۶ سال</x:v>
       </x:c>
-      <x:c r="J16" s="32" t="n">
-        <x:v>48</x:v>
-      </x:c>
-      <x:c r="K16" s="32" t="n">
-        <x:v>84</x:v>
+      <x:c r="J16" s="32" t="str">
+        <x:v>۴ سال</x:v>
+      </x:c>
+      <x:c r="K16" s="32" t="str">
+        <x:v>۷ سال</x:v>
       </x:c>
       <x:c r="L16" s="32" t="n">
         <x:v>8</x:v>
@@ -2706,11 +2706,11 @@
       <x:c r="I17" s="32" t="str">
         <x:v>۴ تا ۶ سال</x:v>
       </x:c>
-      <x:c r="J17" s="32" t="n">
-        <x:v>48</x:v>
-      </x:c>
-      <x:c r="K17" s="32" t="n">
-        <x:v>84</x:v>
+      <x:c r="J17" s="32" t="str">
+        <x:v>۴ سال</x:v>
+      </x:c>
+      <x:c r="K17" s="32" t="str">
+        <x:v>۷ سال</x:v>
       </x:c>
       <x:c r="L17" s="32" t="n">
         <x:v>8</x:v>
@@ -2850,11 +2850,11 @@
       <x:c r="I18" s="32" t="str">
         <x:v>۴ تا ۶ سال</x:v>
       </x:c>
-      <x:c r="J18" s="32" t="n">
-        <x:v>48</x:v>
-      </x:c>
-      <x:c r="K18" s="32" t="n">
-        <x:v>84</x:v>
+      <x:c r="J18" s="32" t="str">
+        <x:v>۴ سال</x:v>
+      </x:c>
+      <x:c r="K18" s="32" t="str">
+        <x:v>۷ سال</x:v>
       </x:c>
       <x:c r="L18" s="32" t="n">
         <x:v>6</x:v>
@@ -2990,11 +2990,11 @@
       <x:c r="I19" s="32" t="str">
         <x:v>۴ تا ۶ سال</x:v>
       </x:c>
-      <x:c r="J19" s="32" t="n">
-        <x:v>48</x:v>
-      </x:c>
-      <x:c r="K19" s="32" t="n">
-        <x:v>84</x:v>
+      <x:c r="J19" s="32" t="str">
+        <x:v>۴ سال</x:v>
+      </x:c>
+      <x:c r="K19" s="32" t="str">
+        <x:v>۷ سال</x:v>
       </x:c>
       <x:c r="L19" s="32" t="n">
         <x:v>6</x:v>
@@ -3136,11 +3136,11 @@
       <x:c r="I20" s="32" t="str">
         <x:v>۷ تا ۹ سال</x:v>
       </x:c>
-      <x:c r="J20" s="32" t="n">
-        <x:v>84</x:v>
-      </x:c>
-      <x:c r="K20" s="32" t="n">
-        <x:v>120</x:v>
+      <x:c r="J20" s="32" t="str">
+        <x:v>۷ سال</x:v>
+      </x:c>
+      <x:c r="K20" s="32" t="str">
+        <x:v>۱۰ سال</x:v>
       </x:c>
       <x:c r="L20" s="32" t="n">
         <x:v>12</x:v>
@@ -3280,11 +3280,11 @@
       <x:c r="I21" s="32" t="str">
         <x:v>۷ تا ۹ سال</x:v>
       </x:c>
-      <x:c r="J21" s="32" t="n">
-        <x:v>84</x:v>
-      </x:c>
-      <x:c r="K21" s="32" t="n">
-        <x:v>120</x:v>
+      <x:c r="J21" s="32" t="str">
+        <x:v>۷ سال</x:v>
+      </x:c>
+      <x:c r="K21" s="32" t="str">
+        <x:v>۱۰ سال</x:v>
       </x:c>
       <x:c r="L21" s="32" t="n">
         <x:v>8</x:v>
@@ -3420,11 +3420,11 @@
       <x:c r="I22" s="32" t="str">
         <x:v>۷ تا ۹ سال</x:v>
       </x:c>
-      <x:c r="J22" s="32" t="n">
-        <x:v>84</x:v>
-      </x:c>
-      <x:c r="K22" s="32" t="n">
-        <x:v>120</x:v>
+      <x:c r="J22" s="32" t="str">
+        <x:v>۷ سال</x:v>
+      </x:c>
+      <x:c r="K22" s="32" t="str">
+        <x:v>۱۰ سال</x:v>
       </x:c>
       <x:c r="L22" s="32" t="n">
         <x:v>12</x:v>
@@ -3564,11 +3564,11 @@
       <x:c r="I23" s="32" t="str">
         <x:v>۷ تا ۹ سال</x:v>
       </x:c>
-      <x:c r="J23" s="32" t="n">
-        <x:v>84</x:v>
-      </x:c>
-      <x:c r="K23" s="32" t="n">
-        <x:v>120</x:v>
+      <x:c r="J23" s="32" t="str">
+        <x:v>۷ سال</x:v>
+      </x:c>
+      <x:c r="K23" s="32" t="str">
+        <x:v>۱۰ سال</x:v>
       </x:c>
       <x:c r="L23" s="32" t="n">
         <x:v>8</x:v>
@@ -3704,11 +3704,11 @@
       <x:c r="I24" s="32" t="str">
         <x:v>۷ تا ۹ سال</x:v>
       </x:c>
-      <x:c r="J24" s="32" t="n">
-        <x:v>84</x:v>
-      </x:c>
-      <x:c r="K24" s="32" t="n">
-        <x:v>120</x:v>
+      <x:c r="J24" s="32" t="str">
+        <x:v>۷ سال</x:v>
+      </x:c>
+      <x:c r="K24" s="32" t="str">
+        <x:v>۱۰ سال</x:v>
       </x:c>
       <x:c r="L24" s="32" t="n">
         <x:v>10</x:v>
@@ -3852,11 +3852,11 @@
       <x:c r="I25" s="32" t="str">
         <x:v>۱۰ تا ۱۲ سال</x:v>
       </x:c>
-      <x:c r="J25" s="32" t="n">
-        <x:v>120</x:v>
-      </x:c>
-      <x:c r="K25" s="32" t="n">
-        <x:v>156</x:v>
+      <x:c r="J25" s="32" t="str">
+        <x:v>۱۰ سال</x:v>
+      </x:c>
+      <x:c r="K25" s="32" t="str">
+        <x:v>۱۲ سال</x:v>
       </x:c>
       <x:c r="L25" s="32" t="n">
         <x:v>10</x:v>
@@ -3992,11 +3992,11 @@
       <x:c r="I26" s="32" t="str">
         <x:v>۱۰ تا ۱۲ سال</x:v>
       </x:c>
-      <x:c r="J26" s="32" t="n">
-        <x:v>120</x:v>
-      </x:c>
-      <x:c r="K26" s="32" t="n">
-        <x:v>156</x:v>
+      <x:c r="J26" s="32" t="str">
+        <x:v>۱۰ سال</x:v>
+      </x:c>
+      <x:c r="K26" s="32" t="str">
+        <x:v>۱۲ سال</x:v>
       </x:c>
       <x:c r="L26" s="32" t="n">
         <x:v>10</x:v>
@@ -4134,11 +4134,11 @@
       <x:c r="I27" s="32" t="str">
         <x:v>۱۰ تا ۱۲ سال</x:v>
       </x:c>
-      <x:c r="J27" s="32" t="n">
-        <x:v>120</x:v>
-      </x:c>
-      <x:c r="K27" s="32" t="n">
-        <x:v>156</x:v>
+      <x:c r="J27" s="32" t="str">
+        <x:v>۱۰ سال</x:v>
+      </x:c>
+      <x:c r="K27" s="32" t="str">
+        <x:v>۱۲ سال</x:v>
       </x:c>
       <x:c r="L27" s="32" t="n">
         <x:v>20</x:v>
@@ -4278,11 +4278,11 @@
       <x:c r="I28" s="32" t="str">
         <x:v>۱۰ تا ۱۲ سال</x:v>
       </x:c>
-      <x:c r="J28" s="32" t="n">
-        <x:v>120</x:v>
-      </x:c>
-      <x:c r="K28" s="32" t="n">
-        <x:v>156</x:v>
+      <x:c r="J28" s="32" t="str">
+        <x:v>۱۰ سال</x:v>
+      </x:c>
+      <x:c r="K28" s="32" t="str">
+        <x:v>۱۲ سال</x:v>
       </x:c>
       <x:c r="L28" s="32" t="n">
         <x:v>10</x:v>
@@ -4418,11 +4418,11 @@
       <x:c r="I29" s="32" t="str">
         <x:v>۱۰ تا ۱۲ سال</x:v>
       </x:c>
-      <x:c r="J29" s="32" t="n">
-        <x:v>120</x:v>
-      </x:c>
-      <x:c r="K29" s="32" t="n">
-        <x:v>156</x:v>
+      <x:c r="J29" s="32" t="str">
+        <x:v>۱۰ سال</x:v>
+      </x:c>
+      <x:c r="K29" s="32" t="str">
+        <x:v>۱۲ سال</x:v>
       </x:c>
       <x:c r="L29" s="32" t="n">
         <x:v>15</x:v>
@@ -4549,6 +4549,12 @@
     </x:dataValidation>
     <x:dataValidation type="list" sqref="I5:I29">
       <x:formula1>"۶ تا ۲۳ ماه,۲ تا ۳ سال,۴ تا ۶ سال,۷ تا ۹ سال,۱۰ تا ۱۲ سال"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="J5:J29">
+      <x:formula1>"۶ ماه,۷ ماه,۸ ماه,۹ ماه,۱۰ ماه,۱۱ ماه,۱۲ ماه,۱ سال,۲ سال,۳ سال,۴ سال,۵ سال,۶ سال,۷ سال,۸ سال,۹ سال,۱۰ سال,۱۱ سال,۱۲ سال"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="K5:K29">
+      <x:formula1>"۶ ماه,۷ ماه,۸ ماه,۹ ماه,۱۰ ماه,۱۱ ماه,۱۲ ماه,۱ سال,۲ سال,۳ سال,۴ سال,۵ سال,۶ سال,۷ سال,۸ سال,۹ سال,۱۰ سال,۱۱ سال,۱۲ سال"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="O5:O29">
       <x:formula1>"روی پا یا بغل,فضای کوچک,اتاق,فضای بزرگ,فضای باز"</x:formula1>
@@ -4640,42 +4646,28 @@
     <x:dataValidation type="list" sqref="BC5:BC29">
       <x:formula1>"در انتظار,تأیید نهایی,نیاز به اصلاح,رد"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="whole" operator="between" sqref="J5:J29">
-      <x:formula1>0</x:formula1>
-      <x:formula2>360</x:formula2>
+    <x:dataValidation type="list" sqref="L5:L29">
+      <x:formula1>"5,10,15,20,30,45,60,90"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="whole" operator="between" sqref="K5:K29">
-      <x:formula1>0</x:formula1>
-      <x:formula2>360</x:formula2>
+    <x:dataValidation type="list" sqref="M5:M29">
+      <x:formula1>"5,10,15,20,30,45,60,90,120"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="whole" operator="between" sqref="L5:L29">
-      <x:formula1>0</x:formula1>
-      <x:formula2>360</x:formula2>
+    <x:dataValidation type="list" sqref="N5:N29">
+      <x:formula1>"0,2,5,10,15,20,30"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="whole" operator="between" sqref="M5:M29">
-      <x:formula1>0</x:formula1>
-      <x:formula2>360</x:formula2>
+    <x:dataValidation type="list" sqref="R5:R29">
+      <x:formula1>"1,2,3,4,5,6,8,10"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="whole" operator="between" sqref="N5:N29">
-      <x:formula1>0</x:formula1>
-      <x:formula2>360</x:formula2>
+    <x:dataValidation type="list" sqref="S5:S29">
+      <x:formula1>"1,2,3,4,5,6,8,10"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="whole" operator="between" sqref="R5:R29">
-      <x:formula1>0</x:formula1>
-      <x:formula2>360</x:formula2>
-    </x:dataValidation>
-    <x:dataValidation type="whole" operator="between" sqref="S5:S29">
-      <x:formula1>0</x:formula1>
-      <x:formula2>360</x:formula2>
-    </x:dataValidation>
-    <x:dataValidation type="whole" operator="between" sqref="T5:T29">
-      <x:formula1>0</x:formula1>
-      <x:formula2>360</x:formula2>
+    <x:dataValidation type="list" sqref="T5:T29">
+      <x:formula1>"0,1,2,3,4,5"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R653577c3313f4fd2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R26d59c2998cf4cb4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>